<commit_message>
Start list: Fix borders
</commit_message>
<xml_diff>
--- a/local/templates/start/StartList.xlsx
+++ b/local/templates/start/StartList.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10909"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/scottgonzalez/Library/Application Support/owlcms/67.4.3+test/local/templates/start/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/scottgonzalez/Library/Application Support/owlcms/67.5.7+quick-start/local/templates/start/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B96E670-7CD5-5D4E-BA42-82582B33AB92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD7D427C-DC62-5149-8E09-3B8C99ADAD9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1540" yWindow="660" windowWidth="33020" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -62,7 +62,17 @@
             <rFont val="Aptos Narrow"/>
             <family val="2"/>
           </rPr>
-          <t>owlcms:verticalBorders(4,1,11)</t>
+          <t xml:space="preserve">owlcms:verticalBorders(4,1,11)
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+          </rPr>
+          <t>owlcms:horizontalBorders(4,1,11)</t>
         </r>
       </text>
     </comment>
@@ -706,7 +716,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -718,6 +728,21 @@
       <left/>
       <right/>
       <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -735,32 +760,32 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1113,19 +1138,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="29" x14ac:dyDescent="0.2">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-      <c r="J1" s="11"/>
-      <c r="K1" s="11"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="6"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="1"/>
@@ -1135,76 +1160,76 @@
       <c r="E2" s="1"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
-      <c r="H2" s="10"/>
-      <c r="I2" s="10"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="G3" s="8" t="s">
+      <c r="G3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="H3" s="8" t="s">
+      <c r="H3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="I3" s="8" t="s">
+      <c r="I3" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="J3" s="8" t="s">
+      <c r="J3" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="K3" s="8" t="s">
+      <c r="K3" s="4" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="H4" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="J4" s="9" t="s">
+      <c r="J4" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="K4" s="4" t="s">
+      <c r="K4" s="11" t="s">
         <v>19</v>
       </c>
     </row>

</xml_diff>